<commit_message>
Show formatting of whole columns and rows in spreadsheets
Empty cells of a coloured or bordered column or row now show its format in .xlsx, .xls and .ods, within the sheet's data. In .ods, repeated empty cells now take each column's own format.
</commit_message>
<xml_diff>
--- a/tests/corpus/xlsx/styles.xlsx
+++ b/tests/corpus/xlsx/styles.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Bold red</t>
   </si>
@@ -62,6 +62,9 @@
   </si>
   <si>
     <t>Neighbour</t>
+  </si>
+  <si>
+    <t>Filled row</t>
   </si>
 </sst>
 </file>
@@ -96,12 +99,17 @@
       <name val="Consolas"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -116,6 +124,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -144,15 +157,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -171,6 +185,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -510,79 +525,91 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="14" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="10" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
       </c>
+      <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="7"/>
+      <c r="C2" s="8"/>
+      <c r="G2" s="1"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="11">
+      <c r="D3" s="12">
         <v>1234.5</v>
       </c>
+      <c r="G3" s="1"/>
     </row>
-    <row r="4" ht="45" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="12" t="s">
+    <row r="4" ht="45" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="16" t="s">
         <v>13</v>
       </c>
+      <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>14</v>
       </c>
+      <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
       <c r="B6" t="s">
         <v>16</v>
+      </c>
+      <c r="G6" s="1"/>
+    </row>
+    <row r="8" spans="1:1" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Show patterned cell fills in spreadsheets
Grey shades are drawn as their blended colour; stripes, grids and crosshatching as lines over the background colour, for .xlsx and .xls.
</commit_message>
<xml_diff>
--- a/tests/corpus/xlsx/styles.xlsx
+++ b/tests/corpus/xlsx/styles.xlsx
@@ -99,7 +99,7 @@
       <name val="Consolas"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -124,6 +124,23 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="lightGray">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="darkTrellis">
+        <fgColor rgb="FFC00000"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="lightHorizontal">
+        <fgColor rgb="FF0070C0"/>
       </patternFill>
     </fill>
     <fill>
@@ -157,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -186,6 +203,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -605,10 +625,13 @@
       <c r="B6" t="s">
         <v>16</v>
       </c>
+      <c r="C6" s="17"/>
+      <c r="D6" s="18"/>
+      <c r="F6" s="19"/>
       <c r="G6" s="1"/>
     </row>
-    <row r="8" spans="1:1" s="17" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
+    <row r="8" spans="1:1" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="20" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>